<commit_message>
Added excel formatting + files movement
</commit_message>
<xml_diff>
--- a/Results/fam_api_test_results.xlsx
+++ b/Results/fam_api_test_results.xlsx
@@ -17,10 +17,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -34,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +50,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,107 +433,132 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>HTTP Method</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Endpoint URL</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Request Headers</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Request Body</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Expected Status Code</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Actual Status Code</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Response Time (ms)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Response Body</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Error Message</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="100" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Test GET User</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>https://jsonplaceholder.typicode.com/users/1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="H2" t="n">
-        <v>528.36</v>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="n">
+        <v>147.69</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>{
   "id": 1,
@@ -540,46 +585,51 @@
 }</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2025-01-24 17:23:20</t>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-27 11:19:32</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="100" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Test POST Create User</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>https://jsonplaceholder.typicode.com/posts</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>{
   "Content-Type": "application/json"
 }</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>{
   "title": "foo",
@@ -588,16 +638,16 @@
 }</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" s="2" t="n">
         <v>201</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" s="2" t="n">
         <v>201</v>
       </c>
-      <c r="H3" t="n">
-        <v>892.3099999999999</v>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="2" t="n">
+        <v>813.34</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>{
   "title": "foo",
@@ -607,19 +657,19 @@
 }</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2025-01-24 17:23:20</t>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-27 11:19:33</t>
         </is>
       </c>
     </row>

</xml_diff>